<commit_message>
fix: no 404 links - redirect not-yet-migrated pages and dead links; import 5 unlisted game pages
- redirects: unmigrated alc.ca pages -> live alc.ca, dead/empty game links -> category page, /fr -> alc.ca French
- link-audit.cjs: offline audit of every internal link in migrated content

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-online-game-detail.report.xlsx
+++ b/tools/importer/reports/import-online-game-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11480" uniqueCount="5724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11530" uniqueCount="5749">
   <si>
     <t>_reportFile</t>
   </si>
@@ -3115,6 +3115,21 @@
     <t>https://www.alc.ca/content/alc/en/play-online/casino/300-shields-extreme.html</t>
   </si>
   <si>
+    <t>en/play-online/casino/5-dragons.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/5-dragons</t>
+  </si>
+  <si>
+    <t>2026-10-20T19:53:25.803Z</t>
+  </si>
+  <si>
+    <t>5 Dragons</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/5-dragons.html</t>
+  </si>
+  <si>
     <t>en/play-online/casino/5-hand-blackjack.report.json</t>
   </si>
   <si>
@@ -3694,6 +3709,36 @@
     <t>https://www.alc.ca/content/alc/en/play-online/casino/big-hot-flaming-pots-tasty-treasures.html</t>
   </si>
   <si>
+    <t>en/play-online/casino/black-diamond-deluxe.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/black-diamond-deluxe</t>
+  </si>
+  <si>
+    <t>2026-10-20T19:53:52.905Z</t>
+  </si>
+  <si>
+    <t>Black Diamond deluxe</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/black-diamond-deluxe.html</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/black-diamond-platinum.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/black-diamond-platinum</t>
+  </si>
+  <si>
+    <t>2026-10-20T19:54:16.028Z</t>
+  </si>
+  <si>
+    <t>Black Diamond Platinum</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/black-diamond-platinum.html</t>
+  </si>
+  <si>
     <t>en/play-online/casino/black-diamond.report.json</t>
   </si>
   <si>
@@ -4384,6 +4429,21 @@
     <t>https://www.alc.ca/content/alc/en/play-online/casino/cash-machine-jackpots.html</t>
   </si>
   <si>
+    <t>en/play-online/casino/cash-machine.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/cash-machine</t>
+  </si>
+  <si>
+    <t>2026-10-20T19:54:04.643Z</t>
+  </si>
+  <si>
+    <t>Cash Machine | Casino Slot Game | Atlantic Lottery</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/cash-machine.html</t>
+  </si>
+  <si>
     <t>en/play-online/casino/cash-melon.report.json</t>
   </si>
   <si>
@@ -6902,6 +6962,21 @@
   </si>
   <si>
     <t>https://www.alc.ca/content/alc/en/play-online/casino/jokrz-wild-jackpot.html</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/jumpin-jack-first-strike.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/jumpin-jack-first-strike</t>
+  </si>
+  <si>
+    <t>2026-10-20T19:53:37.992Z</t>
+  </si>
+  <si>
+    <t>Jumpin Jack First Strike</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/jumpin-jack-first-strike.html</t>
   </si>
   <si>
     <t>en/play-online/casino/key-to-success.report.json</t>
@@ -17577,7 +17652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1148"/>
+  <dimension ref="A1:J1153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -24332,15 +24407,15 @@
         <v>1044</v>
       </c>
       <c r="I211" t="s">
-        <v>507</v>
+        <v>1045</v>
       </c>
       <c r="J211" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B212" t="s">
         <v>991</v>
@@ -24352,7 +24427,7 @@
         <v>12</v>
       </c>
       <c r="E212" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F212" t="s">
         <v>14</v>
@@ -24361,10 +24436,10 @@
         <v>993</v>
       </c>
       <c r="H212" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="I212" t="s">
-        <v>1049</v>
+        <v>507</v>
       </c>
       <c r="J212" t="s">
         <v>1050</v>
@@ -25420,15 +25495,15 @@
         <v>1213</v>
       </c>
       <c r="I245" t="s">
-        <v>543</v>
+        <v>1214</v>
       </c>
       <c r="J245" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="B246" t="s">
         <v>991</v>
@@ -25440,7 +25515,7 @@
         <v>12</v>
       </c>
       <c r="E246" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="F246" t="s">
         <v>14</v>
@@ -25449,10 +25524,10 @@
         <v>993</v>
       </c>
       <c r="H246" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="I246" t="s">
-        <v>1218</v>
+        <v>543</v>
       </c>
       <c r="J246" t="s">
         <v>1219</v>
@@ -26999,135 +27074,135 @@
         <v>1460</v>
       </c>
       <c r="B295" t="s">
+        <v>991</v>
+      </c>
+      <c r="C295" t="s">
+        <v>12</v>
+      </c>
+      <c r="D295" t="s">
+        <v>12</v>
+      </c>
+      <c r="E295" t="s">
         <v>1461</v>
       </c>
-      <c r="C295" t="s">
-        <v>12</v>
-      </c>
-      <c r="D295" t="s">
-        <v>12</v>
-      </c>
-      <c r="E295" t="s">
+      <c r="F295" t="s">
+        <v>14</v>
+      </c>
+      <c r="G295" t="s">
+        <v>993</v>
+      </c>
+      <c r="H295" t="s">
         <v>1462</v>
       </c>
-      <c r="F295" t="s">
-        <v>14</v>
-      </c>
-      <c r="G295" t="s">
-        <v>993</v>
-      </c>
-      <c r="H295" t="s">
+      <c r="I295" t="s">
         <v>1463</v>
       </c>
-      <c r="I295" t="s">
+      <c r="J295" t="s">
         <v>1464</v>
-      </c>
-      <c r="J295" t="s">
-        <v>1465</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
+        <v>1465</v>
+      </c>
+      <c r="B296" t="s">
+        <v>991</v>
+      </c>
+      <c r="C296" t="s">
+        <v>12</v>
+      </c>
+      <c r="D296" t="s">
+        <v>12</v>
+      </c>
+      <c r="E296" t="s">
         <v>1466</v>
       </c>
-      <c r="B296" t="s">
-        <v>991</v>
-      </c>
-      <c r="C296" t="s">
-        <v>12</v>
-      </c>
-      <c r="D296" t="s">
-        <v>12</v>
-      </c>
-      <c r="E296" t="s">
+      <c r="F296" t="s">
+        <v>14</v>
+      </c>
+      <c r="G296" t="s">
+        <v>993</v>
+      </c>
+      <c r="H296" t="s">
         <v>1467</v>
       </c>
-      <c r="F296" t="s">
-        <v>14</v>
-      </c>
-      <c r="G296" t="s">
-        <v>993</v>
-      </c>
-      <c r="H296" t="s">
+      <c r="I296" t="s">
         <v>1468</v>
       </c>
-      <c r="I296" t="s">
+      <c r="J296" t="s">
         <v>1469</v>
-      </c>
-      <c r="J296" t="s">
-        <v>1470</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B297" t="s">
+        <v>991</v>
+      </c>
+      <c r="C297" t="s">
+        <v>12</v>
+      </c>
+      <c r="D297" t="s">
+        <v>12</v>
+      </c>
+      <c r="E297" t="s">
         <v>1471</v>
       </c>
-      <c r="B297" t="s">
-        <v>991</v>
-      </c>
-      <c r="C297" t="s">
-        <v>12</v>
-      </c>
-      <c r="D297" t="s">
-        <v>12</v>
-      </c>
-      <c r="E297" t="s">
+      <c r="F297" t="s">
+        <v>14</v>
+      </c>
+      <c r="G297" t="s">
+        <v>993</v>
+      </c>
+      <c r="H297" t="s">
         <v>1472</v>
       </c>
-      <c r="F297" t="s">
-        <v>14</v>
-      </c>
-      <c r="G297" t="s">
-        <v>993</v>
-      </c>
-      <c r="H297" t="s">
+      <c r="I297" t="s">
         <v>1473</v>
       </c>
-      <c r="I297" t="s">
+      <c r="J297" t="s">
         <v>1474</v>
-      </c>
-      <c r="J297" t="s">
-        <v>1475</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
+        <v>1475</v>
+      </c>
+      <c r="B298" t="s">
+        <v>991</v>
+      </c>
+      <c r="C298" t="s">
+        <v>12</v>
+      </c>
+      <c r="D298" t="s">
+        <v>12</v>
+      </c>
+      <c r="E298" t="s">
         <v>1476</v>
       </c>
-      <c r="B298" t="s">
-        <v>991</v>
-      </c>
-      <c r="C298" t="s">
-        <v>12</v>
-      </c>
-      <c r="D298" t="s">
-        <v>12</v>
-      </c>
-      <c r="E298" t="s">
+      <c r="F298" t="s">
+        <v>14</v>
+      </c>
+      <c r="G298" t="s">
+        <v>993</v>
+      </c>
+      <c r="H298" t="s">
         <v>1477</v>
       </c>
-      <c r="F298" t="s">
-        <v>14</v>
-      </c>
-      <c r="G298" t="s">
-        <v>993</v>
-      </c>
-      <c r="H298" t="s">
+      <c r="I298" t="s">
         <v>1478</v>
       </c>
-      <c r="I298" t="s">
+      <c r="J298" t="s">
         <v>1479</v>
-      </c>
-      <c r="J298" t="s">
-        <v>1480</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B299" t="s">
         <v>1481</v>
-      </c>
-      <c r="B299" t="s">
-        <v>991</v>
       </c>
       <c r="C299" t="s">
         <v>12</v>
@@ -27223,135 +27298,135 @@
         <v>1496</v>
       </c>
       <c r="B302" t="s">
+        <v>991</v>
+      </c>
+      <c r="C302" t="s">
+        <v>12</v>
+      </c>
+      <c r="D302" t="s">
+        <v>12</v>
+      </c>
+      <c r="E302" t="s">
         <v>1497</v>
       </c>
-      <c r="C302" t="s">
-        <v>12</v>
-      </c>
-      <c r="D302" t="s">
-        <v>12</v>
-      </c>
-      <c r="E302" t="s">
+      <c r="F302" t="s">
+        <v>14</v>
+      </c>
+      <c r="G302" t="s">
+        <v>993</v>
+      </c>
+      <c r="H302" t="s">
         <v>1498</v>
       </c>
-      <c r="F302" t="s">
-        <v>14</v>
-      </c>
-      <c r="G302" t="s">
-        <v>993</v>
-      </c>
-      <c r="H302" t="s">
+      <c r="I302" t="s">
         <v>1499</v>
       </c>
-      <c r="I302" t="s">
+      <c r="J302" t="s">
         <v>1500</v>
-      </c>
-      <c r="J302" t="s">
-        <v>1501</v>
       </c>
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B303" t="s">
+        <v>991</v>
+      </c>
+      <c r="C303" t="s">
+        <v>12</v>
+      </c>
+      <c r="D303" t="s">
+        <v>12</v>
+      </c>
+      <c r="E303" t="s">
         <v>1502</v>
       </c>
-      <c r="B303" t="s">
-        <v>991</v>
-      </c>
-      <c r="C303" t="s">
-        <v>12</v>
-      </c>
-      <c r="D303" t="s">
-        <v>12</v>
-      </c>
-      <c r="E303" t="s">
+      <c r="F303" t="s">
+        <v>14</v>
+      </c>
+      <c r="G303" t="s">
+        <v>993</v>
+      </c>
+      <c r="H303" t="s">
         <v>1503</v>
       </c>
-      <c r="F303" t="s">
-        <v>14</v>
-      </c>
-      <c r="G303" t="s">
-        <v>993</v>
-      </c>
-      <c r="H303" t="s">
+      <c r="I303" t="s">
         <v>1504</v>
       </c>
-      <c r="I303" t="s">
+      <c r="J303" t="s">
         <v>1505</v>
-      </c>
-      <c r="J303" t="s">
-        <v>1506</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B304" t="s">
+        <v>991</v>
+      </c>
+      <c r="C304" t="s">
+        <v>12</v>
+      </c>
+      <c r="D304" t="s">
+        <v>12</v>
+      </c>
+      <c r="E304" t="s">
         <v>1507</v>
       </c>
-      <c r="B304" t="s">
-        <v>991</v>
-      </c>
-      <c r="C304" t="s">
-        <v>12</v>
-      </c>
-      <c r="D304" t="s">
-        <v>12</v>
-      </c>
-      <c r="E304" t="s">
+      <c r="F304" t="s">
+        <v>14</v>
+      </c>
+      <c r="G304" t="s">
+        <v>993</v>
+      </c>
+      <c r="H304" t="s">
         <v>1508</v>
       </c>
-      <c r="F304" t="s">
-        <v>14</v>
-      </c>
-      <c r="G304" t="s">
-        <v>993</v>
-      </c>
-      <c r="H304" t="s">
+      <c r="I304" t="s">
         <v>1509</v>
       </c>
-      <c r="I304" t="s">
+      <c r="J304" t="s">
         <v>1510</v>
-      </c>
-      <c r="J304" t="s">
-        <v>1511</v>
       </c>
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B305" t="s">
+        <v>991</v>
+      </c>
+      <c r="C305" t="s">
+        <v>12</v>
+      </c>
+      <c r="D305" t="s">
+        <v>12</v>
+      </c>
+      <c r="E305" t="s">
         <v>1512</v>
       </c>
-      <c r="B305" t="s">
-        <v>991</v>
-      </c>
-      <c r="C305" t="s">
-        <v>12</v>
-      </c>
-      <c r="D305" t="s">
-        <v>12</v>
-      </c>
-      <c r="E305" t="s">
+      <c r="F305" t="s">
+        <v>14</v>
+      </c>
+      <c r="G305" t="s">
+        <v>993</v>
+      </c>
+      <c r="H305" t="s">
         <v>1513</v>
       </c>
-      <c r="F305" t="s">
-        <v>14</v>
-      </c>
-      <c r="G305" t="s">
-        <v>993</v>
-      </c>
-      <c r="H305" t="s">
+      <c r="I305" t="s">
         <v>1514</v>
       </c>
-      <c r="I305" t="s">
+      <c r="J305" t="s">
         <v>1515</v>
-      </c>
-      <c r="J305" t="s">
-        <v>1516</v>
       </c>
     </row>
     <row r="306" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B306" t="s">
         <v>1517</v>
-      </c>
-      <c r="B306" t="s">
-        <v>991</v>
       </c>
       <c r="C306" t="s">
         <v>12</v>
@@ -30444,15 +30519,15 @@
         <v>1999</v>
       </c>
       <c r="I402" t="s">
-        <v>678</v>
+        <v>2000</v>
       </c>
       <c r="J402" t="s">
-        <v>2000</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="403" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B403" t="s">
         <v>991</v>
@@ -30464,7 +30539,7 @@
         <v>12</v>
       </c>
       <c r="E403" t="s">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F403" t="s">
         <v>14</v>
@@ -30473,18 +30548,18 @@
         <v>993</v>
       </c>
       <c r="H403" t="s">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="I403" t="s">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="J403" t="s">
-        <v>2005</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="404" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="B404" t="s">
         <v>991</v>
@@ -30496,7 +30571,7 @@
         <v>12</v>
       </c>
       <c r="E404" t="s">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F404" t="s">
         <v>14</v>
@@ -30505,18 +30580,18 @@
         <v>993</v>
       </c>
       <c r="H404" t="s">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="I404" t="s">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="J404" t="s">
-        <v>2010</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="405" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B405" t="s">
         <v>991</v>
@@ -30528,7 +30603,7 @@
         <v>12</v>
       </c>
       <c r="E405" t="s">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F405" t="s">
         <v>14</v>
@@ -30537,18 +30612,18 @@
         <v>993</v>
       </c>
       <c r="H405" t="s">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="I405" t="s">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="J405" t="s">
-        <v>2015</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="406" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B406" t="s">
         <v>991</v>
@@ -30560,7 +30635,7 @@
         <v>12</v>
       </c>
       <c r="E406" t="s">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F406" t="s">
         <v>14</v>
@@ -30569,10 +30644,10 @@
         <v>993</v>
       </c>
       <c r="H406" t="s">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="I406" t="s">
-        <v>2019</v>
+        <v>678</v>
       </c>
       <c r="J406" t="s">
         <v>2020</v>
@@ -31308,15 +31383,15 @@
         <v>2133</v>
       </c>
       <c r="I429" t="s">
-        <v>713</v>
+        <v>2134</v>
       </c>
       <c r="J429" t="s">
-        <v>2134</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="430" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>2135</v>
+        <v>2136</v>
       </c>
       <c r="B430" t="s">
         <v>991</v>
@@ -31328,7 +31403,7 @@
         <v>12</v>
       </c>
       <c r="E430" t="s">
-        <v>2136</v>
+        <v>2137</v>
       </c>
       <c r="F430" t="s">
         <v>14</v>
@@ -31337,18 +31412,18 @@
         <v>993</v>
       </c>
       <c r="H430" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="I430" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="J430" t="s">
-        <v>2139</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="431" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>2140</v>
+        <v>2141</v>
       </c>
       <c r="B431" t="s">
         <v>991</v>
@@ -31360,7 +31435,7 @@
         <v>12</v>
       </c>
       <c r="E431" t="s">
-        <v>2141</v>
+        <v>2142</v>
       </c>
       <c r="F431" t="s">
         <v>14</v>
@@ -31369,18 +31444,18 @@
         <v>993</v>
       </c>
       <c r="H431" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="I431" t="s">
-        <v>2143</v>
+        <v>2144</v>
       </c>
       <c r="J431" t="s">
-        <v>2144</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="432" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>2145</v>
+        <v>2146</v>
       </c>
       <c r="B432" t="s">
         <v>991</v>
@@ -31392,7 +31467,7 @@
         <v>12</v>
       </c>
       <c r="E432" t="s">
-        <v>2146</v>
+        <v>2147</v>
       </c>
       <c r="F432" t="s">
         <v>14</v>
@@ -31401,18 +31476,18 @@
         <v>993</v>
       </c>
       <c r="H432" t="s">
-        <v>2147</v>
+        <v>2148</v>
       </c>
       <c r="I432" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="J432" t="s">
-        <v>2149</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="433" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>2150</v>
+        <v>2151</v>
       </c>
       <c r="B433" t="s">
         <v>991</v>
@@ -31424,7 +31499,7 @@
         <v>12</v>
       </c>
       <c r="E433" t="s">
-        <v>2151</v>
+        <v>2152</v>
       </c>
       <c r="F433" t="s">
         <v>14</v>
@@ -31433,10 +31508,10 @@
         <v>993</v>
       </c>
       <c r="H433" t="s">
-        <v>2152</v>
+        <v>2153</v>
       </c>
       <c r="I433" t="s">
-        <v>2153</v>
+        <v>713</v>
       </c>
       <c r="J433" t="s">
         <v>2154</v>
@@ -33644,15 +33719,15 @@
         <v>2497</v>
       </c>
       <c r="I502" t="s">
-        <v>738</v>
+        <v>2498</v>
       </c>
       <c r="J502" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="503" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="B503" t="s">
         <v>991</v>
@@ -33664,7 +33739,7 @@
         <v>12</v>
       </c>
       <c r="E503" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="F503" t="s">
         <v>14</v>
@@ -33673,18 +33748,18 @@
         <v>993</v>
       </c>
       <c r="H503" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
       <c r="I503" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="J503" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="504" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="B504" t="s">
         <v>991</v>
@@ -33696,7 +33771,7 @@
         <v>12</v>
       </c>
       <c r="E504" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="F504" t="s">
         <v>14</v>
@@ -33705,18 +33780,18 @@
         <v>993</v>
       </c>
       <c r="H504" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
       <c r="I504" t="s">
-        <v>2507</v>
+        <v>2508</v>
       </c>
       <c r="J504" t="s">
-        <v>2508</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="505" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="B505" t="s">
         <v>991</v>
@@ -33728,7 +33803,7 @@
         <v>12</v>
       </c>
       <c r="E505" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
       <c r="F505" t="s">
         <v>14</v>
@@ -33737,18 +33812,18 @@
         <v>993</v>
       </c>
       <c r="H505" t="s">
-        <v>2511</v>
+        <v>2512</v>
       </c>
       <c r="I505" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
       <c r="J505" t="s">
-        <v>2513</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="506" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>2514</v>
+        <v>2515</v>
       </c>
       <c r="B506" t="s">
         <v>991</v>
@@ -33760,7 +33835,7 @@
         <v>12</v>
       </c>
       <c r="E506" t="s">
-        <v>2515</v>
+        <v>2516</v>
       </c>
       <c r="F506" t="s">
         <v>14</v>
@@ -33769,18 +33844,18 @@
         <v>993</v>
       </c>
       <c r="H506" t="s">
-        <v>2516</v>
+        <v>2517</v>
       </c>
       <c r="I506" t="s">
-        <v>2517</v>
+        <v>2518</v>
       </c>
       <c r="J506" t="s">
-        <v>2518</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="507" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>2519</v>
+        <v>2520</v>
       </c>
       <c r="B507" t="s">
         <v>991</v>
@@ -33792,7 +33867,7 @@
         <v>12</v>
       </c>
       <c r="E507" t="s">
-        <v>2520</v>
+        <v>2521</v>
       </c>
       <c r="F507" t="s">
         <v>14</v>
@@ -33801,10 +33876,10 @@
         <v>993</v>
       </c>
       <c r="H507" t="s">
-        <v>2521</v>
+        <v>2522</v>
       </c>
       <c r="I507" t="s">
-        <v>2522</v>
+        <v>738</v>
       </c>
       <c r="J507" t="s">
         <v>2523</v>
@@ -35724,15 +35799,15 @@
         <v>2821</v>
       </c>
       <c r="I567" t="s">
-        <v>788</v>
+        <v>2822</v>
       </c>
       <c r="J567" t="s">
-        <v>2822</v>
+        <v>2823</v>
       </c>
     </row>
     <row r="568" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A568" t="s">
-        <v>2823</v>
+        <v>2824</v>
       </c>
       <c r="B568" t="s">
         <v>991</v>
@@ -35744,7 +35819,7 @@
         <v>12</v>
       </c>
       <c r="E568" t="s">
-        <v>2824</v>
+        <v>2825</v>
       </c>
       <c r="F568" t="s">
         <v>14</v>
@@ -35753,18 +35828,18 @@
         <v>993</v>
       </c>
       <c r="H568" t="s">
-        <v>2825</v>
+        <v>2826</v>
       </c>
       <c r="I568" t="s">
-        <v>2826</v>
+        <v>2827</v>
       </c>
       <c r="J568" t="s">
-        <v>2827</v>
+        <v>2828</v>
       </c>
     </row>
     <row r="569" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A569" t="s">
-        <v>2828</v>
+        <v>2829</v>
       </c>
       <c r="B569" t="s">
         <v>991</v>
@@ -35776,7 +35851,7 @@
         <v>12</v>
       </c>
       <c r="E569" t="s">
-        <v>2829</v>
+        <v>2830</v>
       </c>
       <c r="F569" t="s">
         <v>14</v>
@@ -35785,18 +35860,18 @@
         <v>993</v>
       </c>
       <c r="H569" t="s">
-        <v>2830</v>
+        <v>2831</v>
       </c>
       <c r="I569" t="s">
-        <v>2831</v>
+        <v>2832</v>
       </c>
       <c r="J569" t="s">
-        <v>2832</v>
+        <v>2833</v>
       </c>
     </row>
     <row r="570" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A570" t="s">
-        <v>2833</v>
+        <v>2834</v>
       </c>
       <c r="B570" t="s">
         <v>991</v>
@@ -35808,7 +35883,7 @@
         <v>12</v>
       </c>
       <c r="E570" t="s">
-        <v>2834</v>
+        <v>2835</v>
       </c>
       <c r="F570" t="s">
         <v>14</v>
@@ -35817,18 +35892,18 @@
         <v>993</v>
       </c>
       <c r="H570" t="s">
-        <v>2835</v>
+        <v>2836</v>
       </c>
       <c r="I570" t="s">
-        <v>2836</v>
+        <v>2837</v>
       </c>
       <c r="J570" t="s">
-        <v>2837</v>
+        <v>2838</v>
       </c>
     </row>
     <row r="571" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A571" t="s">
-        <v>2838</v>
+        <v>2839</v>
       </c>
       <c r="B571" t="s">
         <v>991</v>
@@ -35840,7 +35915,7 @@
         <v>12</v>
       </c>
       <c r="E571" t="s">
-        <v>2839</v>
+        <v>2840</v>
       </c>
       <c r="F571" t="s">
         <v>14</v>
@@ -35849,18 +35924,18 @@
         <v>993</v>
       </c>
       <c r="H571" t="s">
-        <v>2840</v>
+        <v>2841</v>
       </c>
       <c r="I571" t="s">
-        <v>2841</v>
+        <v>2842</v>
       </c>
       <c r="J571" t="s">
-        <v>2842</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="572" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A572" t="s">
-        <v>2843</v>
+        <v>2844</v>
       </c>
       <c r="B572" t="s">
         <v>991</v>
@@ -35872,7 +35947,7 @@
         <v>12</v>
       </c>
       <c r="E572" t="s">
-        <v>2844</v>
+        <v>2845</v>
       </c>
       <c r="F572" t="s">
         <v>14</v>
@@ -35881,10 +35956,10 @@
         <v>993</v>
       </c>
       <c r="H572" t="s">
-        <v>2845</v>
+        <v>2846</v>
       </c>
       <c r="I572" t="s">
-        <v>2846</v>
+        <v>788</v>
       </c>
       <c r="J572" t="s">
         <v>2847</v>
@@ -35980,15 +36055,15 @@
         <v>2860</v>
       </c>
       <c r="I575" t="s">
-        <v>803</v>
+        <v>2861</v>
       </c>
       <c r="J575" t="s">
-        <v>2861</v>
+        <v>2862</v>
       </c>
     </row>
     <row r="576" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A576" t="s">
-        <v>2862</v>
+        <v>2863</v>
       </c>
       <c r="B576" t="s">
         <v>991</v>
@@ -36000,7 +36075,7 @@
         <v>12</v>
       </c>
       <c r="E576" t="s">
-        <v>2863</v>
+        <v>2864</v>
       </c>
       <c r="F576" t="s">
         <v>14</v>
@@ -36009,18 +36084,18 @@
         <v>993</v>
       </c>
       <c r="H576" t="s">
-        <v>2864</v>
+        <v>2865</v>
       </c>
       <c r="I576" t="s">
-        <v>2865</v>
+        <v>2866</v>
       </c>
       <c r="J576" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="577" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A577" t="s">
-        <v>2867</v>
+        <v>2868</v>
       </c>
       <c r="B577" t="s">
         <v>991</v>
@@ -36032,7 +36107,7 @@
         <v>12</v>
       </c>
       <c r="E577" t="s">
-        <v>2868</v>
+        <v>2869</v>
       </c>
       <c r="F577" t="s">
         <v>14</v>
@@ -36041,18 +36116,18 @@
         <v>993</v>
       </c>
       <c r="H577" t="s">
-        <v>2869</v>
+        <v>2870</v>
       </c>
       <c r="I577" t="s">
-        <v>2870</v>
+        <v>2871</v>
       </c>
       <c r="J577" t="s">
-        <v>2871</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="578" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A578" t="s">
-        <v>2872</v>
+        <v>2873</v>
       </c>
       <c r="B578" t="s">
         <v>991</v>
@@ -36064,7 +36139,7 @@
         <v>12</v>
       </c>
       <c r="E578" t="s">
-        <v>2873</v>
+        <v>2874</v>
       </c>
       <c r="F578" t="s">
         <v>14</v>
@@ -36073,18 +36148,18 @@
         <v>993</v>
       </c>
       <c r="H578" t="s">
-        <v>2874</v>
+        <v>2875</v>
       </c>
       <c r="I578" t="s">
-        <v>2875</v>
+        <v>2876</v>
       </c>
       <c r="J578" t="s">
-        <v>2876</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="579" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A579" t="s">
-        <v>2877</v>
+        <v>2878</v>
       </c>
       <c r="B579" t="s">
         <v>991</v>
@@ -36096,7 +36171,7 @@
         <v>12</v>
       </c>
       <c r="E579" t="s">
-        <v>2878</v>
+        <v>2879</v>
       </c>
       <c r="F579" t="s">
         <v>14</v>
@@ -36105,18 +36180,18 @@
         <v>993</v>
       </c>
       <c r="H579" t="s">
-        <v>2879</v>
+        <v>2880</v>
       </c>
       <c r="I579" t="s">
-        <v>2880</v>
+        <v>2881</v>
       </c>
       <c r="J579" t="s">
-        <v>2881</v>
+        <v>2882</v>
       </c>
     </row>
     <row r="580" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A580" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
       <c r="B580" t="s">
         <v>991</v>
@@ -36128,7 +36203,7 @@
         <v>12</v>
       </c>
       <c r="E580" t="s">
-        <v>2883</v>
+        <v>2884</v>
       </c>
       <c r="F580" t="s">
         <v>14</v>
@@ -36137,10 +36212,10 @@
         <v>993</v>
       </c>
       <c r="H580" t="s">
-        <v>2884</v>
+        <v>2885</v>
       </c>
       <c r="I580" t="s">
-        <v>2885</v>
+        <v>803</v>
       </c>
       <c r="J580" t="s">
         <v>2886</v>
@@ -37879,7 +37954,7 @@
         <v>3157</v>
       </c>
       <c r="B635" t="s">
-        <v>1461</v>
+        <v>991</v>
       </c>
       <c r="C635" t="s">
         <v>12</v>
@@ -38039,7 +38114,7 @@
         <v>3182</v>
       </c>
       <c r="B640" t="s">
-        <v>991</v>
+        <v>1481</v>
       </c>
       <c r="C640" t="s">
         <v>12</v>
@@ -40108,15 +40183,15 @@
         <v>3504</v>
       </c>
       <c r="I704" t="s">
-        <v>928</v>
+        <v>3505</v>
       </c>
       <c r="J704" t="s">
-        <v>3505</v>
+        <v>3506</v>
       </c>
     </row>
     <row r="705" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A705" t="s">
-        <v>3506</v>
+        <v>3507</v>
       </c>
       <c r="B705" t="s">
         <v>991</v>
@@ -40128,7 +40203,7 @@
         <v>12</v>
       </c>
       <c r="E705" t="s">
-        <v>3507</v>
+        <v>3508</v>
       </c>
       <c r="F705" t="s">
         <v>14</v>
@@ -40137,18 +40212,18 @@
         <v>993</v>
       </c>
       <c r="H705" t="s">
-        <v>3508</v>
+        <v>3509</v>
       </c>
       <c r="I705" t="s">
-        <v>3509</v>
+        <v>3510</v>
       </c>
       <c r="J705" t="s">
-        <v>3510</v>
+        <v>3511</v>
       </c>
     </row>
     <row r="706" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A706" t="s">
-        <v>3511</v>
+        <v>3512</v>
       </c>
       <c r="B706" t="s">
         <v>991</v>
@@ -40160,7 +40235,7 @@
         <v>12</v>
       </c>
       <c r="E706" t="s">
-        <v>3512</v>
+        <v>3513</v>
       </c>
       <c r="F706" t="s">
         <v>14</v>
@@ -40169,18 +40244,18 @@
         <v>993</v>
       </c>
       <c r="H706" t="s">
-        <v>3513</v>
+        <v>3514</v>
       </c>
       <c r="I706" t="s">
-        <v>3514</v>
+        <v>3515</v>
       </c>
       <c r="J706" t="s">
-        <v>3515</v>
+        <v>3516</v>
       </c>
     </row>
     <row r="707" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A707" t="s">
-        <v>3516</v>
+        <v>3517</v>
       </c>
       <c r="B707" t="s">
         <v>991</v>
@@ -40192,7 +40267,7 @@
         <v>12</v>
       </c>
       <c r="E707" t="s">
-        <v>3517</v>
+        <v>3518</v>
       </c>
       <c r="F707" t="s">
         <v>14</v>
@@ -40201,18 +40276,18 @@
         <v>993</v>
       </c>
       <c r="H707" t="s">
-        <v>3518</v>
+        <v>3519</v>
       </c>
       <c r="I707" t="s">
-        <v>3519</v>
+        <v>3520</v>
       </c>
       <c r="J707" t="s">
-        <v>3520</v>
+        <v>3521</v>
       </c>
     </row>
     <row r="708" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A708" t="s">
-        <v>3521</v>
+        <v>3522</v>
       </c>
       <c r="B708" t="s">
         <v>991</v>
@@ -40224,7 +40299,7 @@
         <v>12</v>
       </c>
       <c r="E708" t="s">
-        <v>3522</v>
+        <v>3523</v>
       </c>
       <c r="F708" t="s">
         <v>14</v>
@@ -40233,18 +40308,18 @@
         <v>993</v>
       </c>
       <c r="H708" t="s">
-        <v>3523</v>
+        <v>3524</v>
       </c>
       <c r="I708" t="s">
-        <v>3524</v>
+        <v>3525</v>
       </c>
       <c r="J708" t="s">
-        <v>3525</v>
+        <v>3526</v>
       </c>
     </row>
     <row r="709" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A709" t="s">
-        <v>3526</v>
+        <v>3527</v>
       </c>
       <c r="B709" t="s">
         <v>991</v>
@@ -40256,7 +40331,7 @@
         <v>12</v>
       </c>
       <c r="E709" t="s">
-        <v>3527</v>
+        <v>3528</v>
       </c>
       <c r="F709" t="s">
         <v>14</v>
@@ -40265,10 +40340,10 @@
         <v>993</v>
       </c>
       <c r="H709" t="s">
-        <v>3528</v>
+        <v>3529</v>
       </c>
       <c r="I709" t="s">
-        <v>3529</v>
+        <v>928</v>
       </c>
       <c r="J709" t="s">
         <v>3530</v>
@@ -40695,7 +40770,7 @@
         <v>3596</v>
       </c>
       <c r="B723" t="s">
-        <v>1461</v>
+        <v>991</v>
       </c>
       <c r="C723" t="s">
         <v>12</v>
@@ -40855,7 +40930,7 @@
         <v>3621</v>
       </c>
       <c r="B728" t="s">
-        <v>991</v>
+        <v>1481</v>
       </c>
       <c r="C728" t="s">
         <v>12</v>
@@ -47575,7 +47650,7 @@
         <v>4671</v>
       </c>
       <c r="B938" t="s">
-        <v>1497</v>
+        <v>991</v>
       </c>
       <c r="C938" t="s">
         <v>12</v>
@@ -47735,7 +47810,7 @@
         <v>4696</v>
       </c>
       <c r="B943" t="s">
-        <v>991</v>
+        <v>1517</v>
       </c>
       <c r="C943" t="s">
         <v>12</v>
@@ -49015,7 +49090,7 @@
         <v>4896</v>
       </c>
       <c r="B983" t="s">
-        <v>1461</v>
+        <v>991</v>
       </c>
       <c r="C983" t="s">
         <v>12</v>
@@ -49175,7 +49250,7 @@
         <v>4921</v>
       </c>
       <c r="B988" t="s">
-        <v>991</v>
+        <v>1481</v>
       </c>
       <c r="C988" t="s">
         <v>12</v>
@@ -49900,15 +49975,15 @@
         <v>5033</v>
       </c>
       <c r="I1010" t="s">
-        <v>237</v>
+        <v>5034</v>
       </c>
       <c r="J1010" t="s">
-        <v>5034</v>
+        <v>5035</v>
       </c>
     </row>
     <row r="1011" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1011" t="s">
-        <v>5035</v>
+        <v>5036</v>
       </c>
       <c r="B1011" t="s">
         <v>991</v>
@@ -49920,7 +49995,7 @@
         <v>12</v>
       </c>
       <c r="E1011" t="s">
-        <v>5036</v>
+        <v>5037</v>
       </c>
       <c r="F1011" t="s">
         <v>14</v>
@@ -49929,18 +50004,18 @@
         <v>993</v>
       </c>
       <c r="H1011" t="s">
-        <v>5037</v>
+        <v>5038</v>
       </c>
       <c r="I1011" t="s">
-        <v>5038</v>
+        <v>5039</v>
       </c>
       <c r="J1011" t="s">
-        <v>5039</v>
+        <v>5040</v>
       </c>
     </row>
     <row r="1012" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1012" t="s">
-        <v>5040</v>
+        <v>5041</v>
       </c>
       <c r="B1012" t="s">
         <v>991</v>
@@ -49952,7 +50027,7 @@
         <v>12</v>
       </c>
       <c r="E1012" t="s">
-        <v>5041</v>
+        <v>5042</v>
       </c>
       <c r="F1012" t="s">
         <v>14</v>
@@ -49961,18 +50036,18 @@
         <v>993</v>
       </c>
       <c r="H1012" t="s">
-        <v>5042</v>
+        <v>5043</v>
       </c>
       <c r="I1012" t="s">
-        <v>5043</v>
+        <v>5044</v>
       </c>
       <c r="J1012" t="s">
-        <v>5044</v>
+        <v>5045</v>
       </c>
     </row>
     <row r="1013" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1013" t="s">
-        <v>5045</v>
+        <v>5046</v>
       </c>
       <c r="B1013" t="s">
         <v>991</v>
@@ -49984,7 +50059,7 @@
         <v>12</v>
       </c>
       <c r="E1013" t="s">
-        <v>5046</v>
+        <v>5047</v>
       </c>
       <c r="F1013" t="s">
         <v>14</v>
@@ -49993,18 +50068,18 @@
         <v>993</v>
       </c>
       <c r="H1013" t="s">
-        <v>5047</v>
+        <v>5048</v>
       </c>
       <c r="I1013" t="s">
-        <v>5048</v>
+        <v>5049</v>
       </c>
       <c r="J1013" t="s">
-        <v>5049</v>
+        <v>5050</v>
       </c>
     </row>
     <row r="1014" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
-        <v>5050</v>
+        <v>5051</v>
       </c>
       <c r="B1014" t="s">
         <v>991</v>
@@ -50016,7 +50091,7 @@
         <v>12</v>
       </c>
       <c r="E1014" t="s">
-        <v>5051</v>
+        <v>5052</v>
       </c>
       <c r="F1014" t="s">
         <v>14</v>
@@ -50025,18 +50100,18 @@
         <v>993</v>
       </c>
       <c r="H1014" t="s">
-        <v>5052</v>
+        <v>5053</v>
       </c>
       <c r="I1014" t="s">
-        <v>5053</v>
+        <v>5054</v>
       </c>
       <c r="J1014" t="s">
-        <v>5054</v>
+        <v>5055</v>
       </c>
     </row>
     <row r="1015" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
-        <v>5055</v>
+        <v>5056</v>
       </c>
       <c r="B1015" t="s">
         <v>991</v>
@@ -50048,7 +50123,7 @@
         <v>12</v>
       </c>
       <c r="E1015" t="s">
-        <v>5056</v>
+        <v>5057</v>
       </c>
       <c r="F1015" t="s">
         <v>14</v>
@@ -50057,10 +50132,10 @@
         <v>993</v>
       </c>
       <c r="H1015" t="s">
-        <v>5057</v>
+        <v>5058</v>
       </c>
       <c r="I1015" t="s">
-        <v>5058</v>
+        <v>237</v>
       </c>
       <c r="J1015" t="s">
         <v>5059</v>
@@ -52844,15 +52919,15 @@
         <v>5492</v>
       </c>
       <c r="I1102" t="s">
-        <v>5488</v>
+        <v>5493</v>
       </c>
       <c r="J1102" t="s">
-        <v>5493</v>
+        <v>5494</v>
       </c>
     </row>
     <row r="1103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1103" t="s">
-        <v>5494</v>
+        <v>5495</v>
       </c>
       <c r="B1103" t="s">
         <v>991</v>
@@ -52864,7 +52939,7 @@
         <v>12</v>
       </c>
       <c r="E1103" t="s">
-        <v>5495</v>
+        <v>5496</v>
       </c>
       <c r="F1103" t="s">
         <v>14</v>
@@ -52873,18 +52948,18 @@
         <v>993</v>
       </c>
       <c r="H1103" t="s">
-        <v>5496</v>
+        <v>5497</v>
       </c>
       <c r="I1103" t="s">
-        <v>5497</v>
+        <v>5498</v>
       </c>
       <c r="J1103" t="s">
-        <v>5498</v>
+        <v>5499</v>
       </c>
     </row>
     <row r="1104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1104" t="s">
-        <v>5499</v>
+        <v>5500</v>
       </c>
       <c r="B1104" t="s">
         <v>991</v>
@@ -52896,7 +52971,7 @@
         <v>12</v>
       </c>
       <c r="E1104" t="s">
-        <v>5500</v>
+        <v>5501</v>
       </c>
       <c r="F1104" t="s">
         <v>14</v>
@@ -52905,18 +52980,18 @@
         <v>993</v>
       </c>
       <c r="H1104" t="s">
-        <v>5501</v>
+        <v>5502</v>
       </c>
       <c r="I1104" t="s">
-        <v>5502</v>
+        <v>5503</v>
       </c>
       <c r="J1104" t="s">
-        <v>5503</v>
+        <v>5504</v>
       </c>
     </row>
     <row r="1105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1105" t="s">
-        <v>5504</v>
+        <v>5505</v>
       </c>
       <c r="B1105" t="s">
         <v>991</v>
@@ -52928,7 +53003,7 @@
         <v>12</v>
       </c>
       <c r="E1105" t="s">
-        <v>5505</v>
+        <v>5506</v>
       </c>
       <c r="F1105" t="s">
         <v>14</v>
@@ -52937,18 +53012,18 @@
         <v>993</v>
       </c>
       <c r="H1105" t="s">
-        <v>5506</v>
+        <v>5507</v>
       </c>
       <c r="I1105" t="s">
-        <v>5507</v>
+        <v>5508</v>
       </c>
       <c r="J1105" t="s">
-        <v>5508</v>
+        <v>5509</v>
       </c>
     </row>
     <row r="1106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1106" t="s">
-        <v>5509</v>
+        <v>5510</v>
       </c>
       <c r="B1106" t="s">
         <v>991</v>
@@ -52960,7 +53035,7 @@
         <v>12</v>
       </c>
       <c r="E1106" t="s">
-        <v>5510</v>
+        <v>5511</v>
       </c>
       <c r="F1106" t="s">
         <v>14</v>
@@ -52969,18 +53044,18 @@
         <v>993</v>
       </c>
       <c r="H1106" t="s">
-        <v>5511</v>
+        <v>5512</v>
       </c>
       <c r="I1106" t="s">
-        <v>5512</v>
+        <v>5513</v>
       </c>
       <c r="J1106" t="s">
-        <v>5513</v>
+        <v>5514</v>
       </c>
     </row>
     <row r="1107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1107" t="s">
-        <v>5514</v>
+        <v>5515</v>
       </c>
       <c r="B1107" t="s">
         <v>991</v>
@@ -52992,7 +53067,7 @@
         <v>12</v>
       </c>
       <c r="E1107" t="s">
-        <v>5515</v>
+        <v>5516</v>
       </c>
       <c r="F1107" t="s">
         <v>14</v>
@@ -53001,10 +53076,10 @@
         <v>993</v>
       </c>
       <c r="H1107" t="s">
-        <v>5516</v>
+        <v>5517</v>
       </c>
       <c r="I1107" t="s">
-        <v>5517</v>
+        <v>5513</v>
       </c>
       <c r="J1107" t="s">
         <v>5518</v>
@@ -54320,6 +54395,166 @@
       </c>
       <c r="J1148" t="s">
         <v>5723</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1149" t="s">
+        <v>5724</v>
+      </c>
+      <c r="B1149" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1149" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1149" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1149" t="s">
+        <v>5725</v>
+      </c>
+      <c r="F1149" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1149" t="s">
+        <v>993</v>
+      </c>
+      <c r="H1149" t="s">
+        <v>5726</v>
+      </c>
+      <c r="I1149" t="s">
+        <v>5727</v>
+      </c>
+      <c r="J1149" t="s">
+        <v>5728</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1150" t="s">
+        <v>5729</v>
+      </c>
+      <c r="B1150" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1150" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1150" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1150" t="s">
+        <v>5730</v>
+      </c>
+      <c r="F1150" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1150" t="s">
+        <v>993</v>
+      </c>
+      <c r="H1150" t="s">
+        <v>5731</v>
+      </c>
+      <c r="I1150" t="s">
+        <v>5732</v>
+      </c>
+      <c r="J1150" t="s">
+        <v>5733</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1151" t="s">
+        <v>5734</v>
+      </c>
+      <c r="B1151" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1151" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1151" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1151" t="s">
+        <v>5735</v>
+      </c>
+      <c r="F1151" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1151" t="s">
+        <v>993</v>
+      </c>
+      <c r="H1151" t="s">
+        <v>5736</v>
+      </c>
+      <c r="I1151" t="s">
+        <v>5737</v>
+      </c>
+      <c r="J1151" t="s">
+        <v>5738</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1152" t="s">
+        <v>5739</v>
+      </c>
+      <c r="B1152" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1152" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1152" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1152" t="s">
+        <v>5740</v>
+      </c>
+      <c r="F1152" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1152" t="s">
+        <v>993</v>
+      </c>
+      <c r="H1152" t="s">
+        <v>5741</v>
+      </c>
+      <c r="I1152" t="s">
+        <v>5742</v>
+      </c>
+      <c r="J1152" t="s">
+        <v>5743</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1153" t="s">
+        <v>5744</v>
+      </c>
+      <c r="B1153" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1153" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1153" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>5745</v>
+      </c>
+      <c r="F1153" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1153" t="s">
+        <v>993</v>
+      </c>
+      <c r="H1153" t="s">
+        <v>5746</v>
+      </c>
+      <c r="I1153" t="s">
+        <v>5747</v>
+      </c>
+      <c r="J1153" t="s">
+        <v>5748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>